<commit_message>
organoid: update manifest papers
</commit_message>
<xml_diff>
--- a/collections/organoid/organoid_protocols_papers.xlsx
+++ b/collections/organoid/organoid_protocols_papers.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2599,6 +2599,486 @@
       <c r="L36" t="inlineStr">
         <is>
           <t>human cerebellar organoid generation and long-term culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Bergmann</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>blood-brain barrier</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2018-10-31</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Blood–brain-barrier organoids for investigating the permeability of CNS therapeutics</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>bergmann_2018_bloodbrain-barrier_organoids_for_investigating_the.pdf</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>raw/sources/bergmann_2018_bloodbrain-barrier_organoids_for_investigating_the.pdf</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>wiki/sources/bergmann_2018_bloodbrain-barrier_organoids_for_investigating_the.md</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-018-0066-x</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-018-0066-x.pdf</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>blood-brain-barrier organoid generation for CNS therapeutic permeability assays</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Dekkers</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>multi-organ imaging</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2019-05-03</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>High-resolution 3D imaging of fixed and cleared organoids</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>dekkers_2019_high-resolution_3d_imaging_of_fixed.pdf</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>raw/sources/dekkers_2019_high-resolution_3d_imaging_of_fixed.pdf</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>wiki/sources/dekkers_2019_high-resolution_3d_imaging_of_fixed.md</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-019-0160-8</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-019-0160-8.pdf</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>whole-organoid clearing and high-resolution 3D imaging workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Tysoe</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>biliary</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2019-05-20</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Isolation and propagation of primary human cholangiocyte organoids for the generation of bioengineered biliary tissue</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>tysoe_2019_isolation_and_propagation_of_primary.pdf</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>raw/sources/tysoe_2019_isolation_and_propagation_of_primary.pdf</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>wiki/sources/tysoe_2019_isolation_and_propagation_of_primary.md</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-019-0168-0</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-019-0168-0.pdf</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>primary human cholangiocyte organoid derivation and bioengineered biliary tissue generation</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sheridan</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>placenta</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2020-09-09</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Establishment and differentiation of long-term trophoblast organoid cultures from the human placenta</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>sheridan_2020_establishment_and_differentiation_of_long-term.pdf</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>raw/sources/sheridan_2020_establishment_and_differentiation_of_long-term.pdf</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>wiki/sources/sheridan_2020_establishment_and_differentiation_of_long-term.md</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-020-0381-x</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-020-0381-x.pdf</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>long-term trophoblast organoid derivation and differentiation from human placenta</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Miura</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>brain assembloid</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2022-01-06</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Engineering brain assembloids to interrogate human neural circuits</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>miura_2022_engineering_brain_assembloids_to_interrogate.pdf</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>raw/sources/miura_2022_engineering_brain_assembloids_to_interrogate.pdf</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>wiki/sources/miura_2022_engineering_brain_assembloids_to_interrogate.md</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-021-00632-z</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-021-00632-z.pdf</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>brain assembloid engineering for long-range connectivity and circuit interrogation</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Bakker</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ductal epithelial organoids + imaging</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2022-02-18</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Preparing ductal epithelial organoids for high-spatial-resolution molecular profiling using mass spectrometry imaging</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>bakker_2022_preparing_ductal_epithelial_organoids_for.pdf</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>raw/sources/bakker_2022_preparing_ductal_epithelial_organoids_for.pdf</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>wiki/sources/bakker_2022_preparing_ductal_epithelial_organoids_for.md</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-021-00661-8</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-021-00661-8.pdf</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>mass spectrometry imaging preparation workflow for ductal epithelial organoids</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Gurumurthy</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>cervix</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2022-05-11</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Patient-derived and mouse endo-ectocervical organoid generation, genetic manipulation and applications to model infection</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>gurumurthy_2022_patient-derived_and_mouse_endo-ectocervical_organoid.pdf</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>raw/sources/gurumurthy_2022_patient-derived_and_mouse_endo-ectocervical_organoid.pdf</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>wiki/sources/gurumurthy_2022_patient-derived_and_mouse_endo-ectocervical_organoid.md</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-022-00695-6</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-022-00695-6.pdf</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>endo-ectocervical organoid derivation, genetic manipulation, and infection modeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>forebrain + eye</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2023-05-17</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Generation of iPSC-derived human forebrain organoids assembling bilateral eye primordia</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>gabriel_2023_generation_of_ipsc-derived_human_forebrain.pdf</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>raw/sources/gabriel_2023_generation_of_ipsc-derived_human_forebrain.pdf</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>wiki/sources/gabriel_2023_generation_of_ipsc-derived_human_forebrain.md</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-023-00814-x</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/articles/s41596-023-00814-x.pdf</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>forebrain organoids with bilateral eye primordia assembly from iPSCs</t>
         </is>
       </c>
     </row>
@@ -2674,6 +3154,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J36" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>